<commit_message>
data: update BWV, KV
</commit_message>
<xml_diff>
--- a/xlsx/BWV.xlsx
+++ b/xlsx/BWV.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21942" windowHeight="9805"/>
+    <workbookView windowWidth="21942" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="BWV" sheetId="1" r:id="rId1"/>
@@ -7799,7 +7799,7 @@
     <t>BWV 912a</t>
   </si>
   <si>
-    <t>Variations sur un mouvement de la Toccata BWV 912</t>
+    <t>Variations on a movement of the Toccata BWV 912</t>
   </si>
   <si>
     <t>BWV 913</t>
@@ -7820,7 +7820,7 @@
     <t>BWV 918</t>
   </si>
   <si>
-    <t>Fantaisie sur un Rondo</t>
+    <t>Fantaisie on a Rondo</t>
   </si>
   <si>
     <t>BWV 919</t>
@@ -8469,7 +8469,7 @@
 4. Presto</t>
   </si>
   <si>
-    <t>Solo Violin solo</t>
+    <t>Solo Violin</t>
   </si>
   <si>
     <t>BWV 1002</t>

</xml_diff>